<commit_message>
BOM with price updated 10 Boards Quantity.
</commit_message>
<xml_diff>
--- a/Design-Files/Mains_Board/Deliverables/BOM/BOM With Price-Mains_Board.xlsx
+++ b/Design-Files/Mains_Board/Deliverables/BOM/BOM With Price-Mains_Board.xlsx
@@ -4,11 +4,12 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView windowWidth="20490" windowHeight="7620" activeTab="1"/>
+    <workbookView windowWidth="20490" windowHeight="7500" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="5 Boards" sheetId="1" r:id="rId1"/>
-    <sheet name="100 Boards" sheetId="2" r:id="rId2"/>
+    <sheet name="10 Boards" sheetId="3" r:id="rId2"/>
+    <sheet name="100 Boards" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="446" uniqueCount="114">
   <si>
     <t>#</t>
   </si>
@@ -346,6 +347,18 @@
   </si>
   <si>
     <t>Single Board Cost</t>
+  </si>
+  <si>
+    <t>Quantity (10 Boards)</t>
+  </si>
+  <si>
+    <t>MOQ (10 Boards)</t>
+  </si>
+  <si>
+    <t>Unit Cost (10 Boards)</t>
+  </si>
+  <si>
+    <t>Total Cost (10 Boards)</t>
   </si>
   <si>
     <t>Quantity (100 Boards)</t>
@@ -372,7 +385,7 @@
     <numFmt numFmtId="178" formatCode="&quot;$&quot;#,##0.0000"/>
     <numFmt numFmtId="179" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="31">
+  <fonts count="30">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -450,13 +463,6 @@
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -1039,148 +1045,148 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="10" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="6" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="8" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="17" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="8" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="17" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1262,17 +1268,17 @@
     <xf numFmtId="179" fontId="9" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="4" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="4" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
@@ -1603,8 +1609,8 @@
   <dimension ref="A1:R29"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="3.14285714285714" style="27" customWidth="1"/>
-    <col min="3" max="3" width="18" style="27" customWidth="1"/>
+    <col min="2" max="2" width="3.14285714285714" style="30" customWidth="1"/>
+    <col min="3" max="3" width="18" style="30" customWidth="1"/>
     <col min="4" max="4" width="27.4285714285714" customWidth="1"/>
     <col min="5" max="5" width="30.8571428571429" customWidth="1"/>
     <col min="6" max="6" width="22.2857142857143" customWidth="1"/>
@@ -1739,7 +1745,7 @@
       <c r="N3" s="9">
         <v>5</v>
       </c>
-      <c r="O3" s="28" t="s">
+      <c r="O3" s="27" t="s">
         <v>26</v>
       </c>
       <c r="P3" s="17">
@@ -1794,7 +1800,7 @@
       <c r="N4" s="12">
         <v>10</v>
       </c>
-      <c r="O4" s="29" t="s">
+      <c r="O4" s="28" t="s">
         <v>26</v>
       </c>
       <c r="P4" s="19">
@@ -1849,7 +1855,7 @@
       <c r="N5" s="9">
         <v>50</v>
       </c>
-      <c r="O5" s="29" t="s">
+      <c r="O5" s="28" t="s">
         <v>26</v>
       </c>
       <c r="P5" s="17">
@@ -1904,7 +1910,7 @@
       <c r="N6" s="12">
         <v>10</v>
       </c>
-      <c r="O6" s="29" t="s">
+      <c r="O6" s="28" t="s">
         <v>26</v>
       </c>
       <c r="P6" s="19">
@@ -1959,7 +1965,7 @@
       <c r="N7" s="9">
         <v>5</v>
       </c>
-      <c r="O7" s="29" t="s">
+      <c r="O7" s="28" t="s">
         <v>26</v>
       </c>
       <c r="P7" s="17">
@@ -2014,7 +2020,7 @@
       <c r="N8" s="12">
         <v>15</v>
       </c>
-      <c r="O8" s="30" t="s">
+      <c r="O8" s="29" t="s">
         <v>59</v>
       </c>
       <c r="P8" s="21">
@@ -2069,7 +2075,7 @@
       <c r="N9" s="9">
         <v>10</v>
       </c>
-      <c r="O9" s="30" t="s">
+      <c r="O9" s="29" t="s">
         <v>65</v>
       </c>
       <c r="P9" s="17">
@@ -2124,7 +2130,7 @@
       <c r="N10" s="12">
         <v>10</v>
       </c>
-      <c r="O10" s="30" t="s">
+      <c r="O10" s="29" t="s">
         <v>26</v>
       </c>
       <c r="P10" s="19">
@@ -2179,7 +2185,7 @@
       <c r="N11" s="9">
         <v>100</v>
       </c>
-      <c r="O11" s="30" t="str">
+      <c r="O11" s="29" t="str">
         <f t="shared" ref="O11" si="9">HYPERLINK(AB11,"LCSC")</f>
         <v>LCSC</v>
       </c>
@@ -2235,7 +2241,7 @@
       <c r="N12" s="12">
         <v>100</v>
       </c>
-      <c r="O12" s="30" t="s">
+      <c r="O12" s="29" t="s">
         <v>26</v>
       </c>
       <c r="P12" s="19">
@@ -2290,7 +2296,7 @@
       <c r="N13" s="9">
         <v>20</v>
       </c>
-      <c r="O13" s="30" t="s">
+      <c r="O13" s="29" t="s">
         <v>26</v>
       </c>
       <c r="P13" s="17">
@@ -2345,7 +2351,7 @@
       <c r="N14" s="12">
         <v>100</v>
       </c>
-      <c r="O14" s="30" t="s">
+      <c r="O14" s="29" t="s">
         <v>26</v>
       </c>
       <c r="P14" s="19">
@@ -2400,7 +2406,7 @@
       <c r="N15" s="9">
         <v>5</v>
       </c>
-      <c r="O15" s="30" t="s">
+      <c r="O15" s="29" t="s">
         <v>26</v>
       </c>
       <c r="P15" s="17">
@@ -2492,6 +2498,895 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:R17"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="3.57142857142857" customWidth="1"/>
+    <col min="3" max="3" width="10.4285714285714" customWidth="1"/>
+    <col min="4" max="4" width="11.2857142857143" customWidth="1"/>
+    <col min="5" max="5" width="28" customWidth="1"/>
+    <col min="6" max="6" width="12.8571428571429" customWidth="1"/>
+    <col min="7" max="7" width="27.2857142857143" customWidth="1"/>
+    <col min="8" max="8" width="14.1428571428571" customWidth="1"/>
+    <col min="9" max="9" width="23.1428571428571" customWidth="1"/>
+    <col min="10" max="10" width="18.2857142857143" customWidth="1"/>
+    <col min="11" max="11" width="6.71428571428571" customWidth="1"/>
+    <col min="12" max="12" width="9.28571428571429" customWidth="1"/>
+    <col min="13" max="13" width="19.5714285714286" customWidth="1"/>
+    <col min="14" max="14" width="16.2857142857143" customWidth="1"/>
+    <col min="15" max="15" width="8.28571428571429" customWidth="1"/>
+    <col min="16" max="16" width="20.1428571428571" customWidth="1"/>
+    <col min="17" max="17" width="20.7142857142857" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="15.75" spans="1:18">
+      <c r="A1" s="2"/>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
+      <c r="H1" s="4"/>
+      <c r="I1" s="4"/>
+      <c r="J1" s="4"/>
+      <c r="K1" s="13"/>
+      <c r="L1" s="13"/>
+      <c r="M1" s="13"/>
+      <c r="N1" s="13"/>
+      <c r="O1" s="13"/>
+      <c r="P1" s="13"/>
+      <c r="Q1" s="13"/>
+      <c r="R1" s="13"/>
+    </row>
+    <row r="2" ht="15.75" spans="1:18">
+      <c r="A2" s="2"/>
+      <c r="B2" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="J2" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="K2" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="L2" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="M2" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="N2" s="14" t="s">
+        <v>107</v>
+      </c>
+      <c r="O2" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="P2" s="15" t="s">
+        <v>108</v>
+      </c>
+      <c r="Q2" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="R2" s="5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18">
+      <c r="A3" s="2"/>
+      <c r="B3" s="7">
+        <f>ROW(B3)-ROW($B$2)</f>
+        <v>1</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="G3" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="H3" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="I3" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="J3" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="K3" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="L3" s="9">
+        <v>1</v>
+      </c>
+      <c r="M3" s="9">
+        <f>L3*10</f>
+        <v>10</v>
+      </c>
+      <c r="N3" s="9">
+        <v>10</v>
+      </c>
+      <c r="O3" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="P3" s="17">
+        <v>0.0985</v>
+      </c>
+      <c r="Q3" s="17">
+        <f t="shared" ref="Q3:Q15" si="0">P3*N3</f>
+        <v>0.985</v>
+      </c>
+      <c r="R3" s="9"/>
+    </row>
+    <row r="4" ht="48" spans="1:18">
+      <c r="A4" s="2"/>
+      <c r="B4" s="10">
+        <f>ROW(B4)-ROW($B$2)</f>
+        <v>2</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="E4" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="F4" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="G4" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="H4" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="I4" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="J4" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="K4" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="L4" s="12">
+        <v>2</v>
+      </c>
+      <c r="M4" s="9">
+        <f t="shared" ref="M4:M15" si="1">L4*10</f>
+        <v>20</v>
+      </c>
+      <c r="N4" s="12">
+        <v>20</v>
+      </c>
+      <c r="O4" s="28" t="s">
+        <v>26</v>
+      </c>
+      <c r="P4" s="19">
+        <v>0.0819</v>
+      </c>
+      <c r="Q4" s="19">
+        <f t="shared" si="0"/>
+        <v>1.638</v>
+      </c>
+      <c r="R4" s="12"/>
+    </row>
+    <row r="5" ht="96" spans="1:18">
+      <c r="A5" s="2"/>
+      <c r="B5" s="7">
+        <f>ROW(B5)-ROW($B$2)</f>
+        <v>3</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="F5" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="G5" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="H5" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="I5" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="J5" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="K5" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="L5" s="9">
+        <v>1</v>
+      </c>
+      <c r="M5" s="9">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="N5" s="9">
+        <v>50</v>
+      </c>
+      <c r="O5" s="28" t="s">
+        <v>26</v>
+      </c>
+      <c r="P5" s="17">
+        <v>0.0081</v>
+      </c>
+      <c r="Q5" s="17">
+        <f t="shared" si="0"/>
+        <v>0.405</v>
+      </c>
+      <c r="R5" s="9"/>
+    </row>
+    <row r="6" ht="48" spans="1:18">
+      <c r="A6" s="2"/>
+      <c r="B6" s="10">
+        <f>ROW(B6)-ROW($B$2)</f>
+        <v>4</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="E6" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="F6" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="G6" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="H6" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="I6" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="J6" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="K6" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="L6" s="12">
+        <v>1</v>
+      </c>
+      <c r="M6" s="9">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="N6" s="12">
+        <v>10</v>
+      </c>
+      <c r="O6" s="28" t="s">
+        <v>26</v>
+      </c>
+      <c r="P6" s="19">
+        <v>0.0448</v>
+      </c>
+      <c r="Q6" s="19">
+        <f t="shared" si="0"/>
+        <v>0.448</v>
+      </c>
+      <c r="R6" s="12"/>
+    </row>
+    <row r="7" ht="180" spans="1:18">
+      <c r="A7" s="2"/>
+      <c r="B7" s="7">
+        <f>ROW(B7)-ROW($B$2)</f>
+        <v>5</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="F7" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="G7" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="H7" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="I7" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="J7" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="K7" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="L7" s="9">
+        <v>1</v>
+      </c>
+      <c r="M7" s="9">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="N7" s="9">
+        <v>10</v>
+      </c>
+      <c r="O7" s="28" t="s">
+        <v>26</v>
+      </c>
+      <c r="P7" s="17">
+        <v>0.1088</v>
+      </c>
+      <c r="Q7" s="17">
+        <f t="shared" si="0"/>
+        <v>1.088</v>
+      </c>
+      <c r="R7" s="9"/>
+    </row>
+    <row r="8" ht="48" spans="1:18">
+      <c r="A8" s="2"/>
+      <c r="B8" s="10">
+        <f>ROW(B8)-ROW($B$2)</f>
+        <v>6</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="E8" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="F8" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="G8" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="H8" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="I8" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="J8" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="K8" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="L8" s="12">
+        <v>3</v>
+      </c>
+      <c r="M8" s="9">
+        <f t="shared" si="1"/>
+        <v>30</v>
+      </c>
+      <c r="N8" s="12">
+        <v>30</v>
+      </c>
+      <c r="O8" s="29" t="s">
+        <v>59</v>
+      </c>
+      <c r="P8" s="21">
+        <v>0.63</v>
+      </c>
+      <c r="Q8" s="19">
+        <f t="shared" si="0"/>
+        <v>18.9</v>
+      </c>
+      <c r="R8" s="12"/>
+    </row>
+    <row r="9" ht="48" spans="1:18">
+      <c r="A9" s="2"/>
+      <c r="B9" s="7">
+        <f>ROW(B9)-ROW($B$2)</f>
+        <v>7</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="E9" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="F9" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="G9" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="H9" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="I9" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="J9" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="K9" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="L9" s="9">
+        <v>2</v>
+      </c>
+      <c r="M9" s="9">
+        <f t="shared" si="1"/>
+        <v>20</v>
+      </c>
+      <c r="N9" s="9">
+        <v>20</v>
+      </c>
+      <c r="O9" s="29" t="s">
+        <v>65</v>
+      </c>
+      <c r="P9" s="17">
+        <v>4.01</v>
+      </c>
+      <c r="Q9" s="17">
+        <f t="shared" si="0"/>
+        <v>80.2</v>
+      </c>
+      <c r="R9" s="9"/>
+    </row>
+    <row r="10" ht="108" spans="1:18">
+      <c r="A10" s="2"/>
+      <c r="B10" s="10">
+        <f>ROW(B10)-ROW($B$2)</f>
+        <v>8</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="D10" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="E10" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="F10" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="G10" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="H10" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="I10" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="J10" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="K10" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="L10" s="12">
+        <v>2</v>
+      </c>
+      <c r="M10" s="9">
+        <f t="shared" si="1"/>
+        <v>20</v>
+      </c>
+      <c r="N10" s="12">
+        <v>10</v>
+      </c>
+      <c r="O10" s="29" t="s">
+        <v>26</v>
+      </c>
+      <c r="P10" s="19">
+        <v>0.0274</v>
+      </c>
+      <c r="Q10" s="19">
+        <f t="shared" si="0"/>
+        <v>0.274</v>
+      </c>
+      <c r="R10" s="12"/>
+    </row>
+    <row r="11" ht="48" spans="1:18">
+      <c r="A11" s="2"/>
+      <c r="B11" s="7">
+        <f>ROW(B11)-ROW($B$2)</f>
+        <v>9</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="F11" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="G11" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="H11" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="I11" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="J11" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="K11" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="L11" s="9">
+        <v>3</v>
+      </c>
+      <c r="M11" s="9">
+        <f t="shared" si="1"/>
+        <v>30</v>
+      </c>
+      <c r="N11" s="9">
+        <v>100</v>
+      </c>
+      <c r="O11" s="29" t="str">
+        <f>HYPERLINK(AB11,"LCSC")</f>
+        <v>LCSC</v>
+      </c>
+      <c r="P11" s="21" t="s">
+        <v>81</v>
+      </c>
+      <c r="Q11" s="17">
+        <f t="shared" si="0"/>
+        <v>0.11</v>
+      </c>
+      <c r="R11" s="9"/>
+    </row>
+    <row r="12" ht="48" spans="1:18">
+      <c r="A12" s="2"/>
+      <c r="B12" s="10">
+        <f>ROW(B12)-ROW($B$2)</f>
+        <v>10</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="D12" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="E12" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="F12" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="G12" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="H12" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="I12" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="J12" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="K12" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="L12" s="12">
+        <v>2</v>
+      </c>
+      <c r="M12" s="9">
+        <f t="shared" si="1"/>
+        <v>20</v>
+      </c>
+      <c r="N12" s="12">
+        <v>100</v>
+      </c>
+      <c r="O12" s="29" t="s">
+        <v>26</v>
+      </c>
+      <c r="P12" s="19">
+        <v>0.0006</v>
+      </c>
+      <c r="Q12" s="19">
+        <f t="shared" si="0"/>
+        <v>0.06</v>
+      </c>
+      <c r="R12" s="12"/>
+    </row>
+    <row r="13" ht="60" spans="1:18">
+      <c r="A13" s="2"/>
+      <c r="B13" s="7">
+        <f>ROW(B13)-ROW($B$2)</f>
+        <v>11</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="D13" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="E13" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="F13" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="G13" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="H13" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="I13" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="J13" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="K13" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="L13" s="9">
+        <v>2</v>
+      </c>
+      <c r="M13" s="9">
+        <f t="shared" si="1"/>
+        <v>20</v>
+      </c>
+      <c r="N13" s="9">
+        <v>20</v>
+      </c>
+      <c r="O13" s="29" t="s">
+        <v>26</v>
+      </c>
+      <c r="P13" s="17">
+        <v>0.0203</v>
+      </c>
+      <c r="Q13" s="17">
+        <f t="shared" si="0"/>
+        <v>0.406</v>
+      </c>
+      <c r="R13" s="9"/>
+    </row>
+    <row r="14" ht="48" spans="1:18">
+      <c r="A14" s="2"/>
+      <c r="B14" s="10">
+        <f>ROW(B14)-ROW($B$2)</f>
+        <v>12</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="D14" s="12" t="s">
+        <v>93</v>
+      </c>
+      <c r="E14" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="F14" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="G14" s="12" t="s">
+        <v>95</v>
+      </c>
+      <c r="H14" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="I14" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="J14" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="K14" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="L14" s="12">
+        <v>2</v>
+      </c>
+      <c r="M14" s="9">
+        <f t="shared" si="1"/>
+        <v>20</v>
+      </c>
+      <c r="N14" s="12">
+        <v>100</v>
+      </c>
+      <c r="O14" s="29" t="s">
+        <v>26</v>
+      </c>
+      <c r="P14" s="19">
+        <v>0.0012</v>
+      </c>
+      <c r="Q14" s="19">
+        <f t="shared" si="0"/>
+        <v>0.12</v>
+      </c>
+      <c r="R14" s="12"/>
+    </row>
+    <row r="15" ht="48.75" spans="1:18">
+      <c r="A15" s="2"/>
+      <c r="B15" s="7">
+        <f>ROW(B15)-ROW($B$2)</f>
+        <v>13</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="E15" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="F15" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="G15" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="H15" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="I15" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="J15" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="K15" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="L15" s="9">
+        <v>1</v>
+      </c>
+      <c r="M15" s="9">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="N15" s="9">
+        <v>10</v>
+      </c>
+      <c r="O15" s="29" t="s">
+        <v>26</v>
+      </c>
+      <c r="P15" s="17">
+        <v>0.4611</v>
+      </c>
+      <c r="Q15" s="17">
+        <f t="shared" si="0"/>
+        <v>4.611</v>
+      </c>
+      <c r="R15" s="9"/>
+    </row>
+    <row r="16" ht="19.5" spans="1:18">
+      <c r="A16" s="2"/>
+      <c r="B16" s="2"/>
+      <c r="C16" s="2"/>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="2"/>
+      <c r="H16" s="2"/>
+      <c r="I16" s="2"/>
+      <c r="J16" s="2"/>
+      <c r="K16" s="2"/>
+      <c r="L16" s="2"/>
+      <c r="M16" s="2"/>
+      <c r="N16" s="23" t="s">
+        <v>104</v>
+      </c>
+      <c r="O16" s="24"/>
+      <c r="P16" s="24"/>
+      <c r="Q16" s="25">
+        <f>SUM(Q3:Q15)</f>
+        <v>109.245</v>
+      </c>
+      <c r="R16" s="2"/>
+    </row>
+    <row r="17" ht="19.5" spans="1:18">
+      <c r="A17" s="2"/>
+      <c r="B17" s="2"/>
+      <c r="C17" s="2"/>
+      <c r="D17" s="2"/>
+      <c r="E17" s="2"/>
+      <c r="F17" s="2"/>
+      <c r="G17" s="2"/>
+      <c r="H17" s="2"/>
+      <c r="I17" s="2"/>
+      <c r="J17" s="2"/>
+      <c r="K17" s="2"/>
+      <c r="L17" s="2"/>
+      <c r="M17" s="2"/>
+      <c r="N17" s="23" t="s">
+        <v>105</v>
+      </c>
+      <c r="O17" s="24"/>
+      <c r="P17" s="24"/>
+      <c r="Q17" s="26">
+        <f>Q16/10</f>
+        <v>10.9245</v>
+      </c>
+      <c r="R17" s="2"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="K1:R1"/>
+    <mergeCell ref="N16:P16"/>
+    <mergeCell ref="N17:P17"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="O8" r:id="rId1" display="Mouser"/>
+    <hyperlink ref="O9" r:id="rId2" display="Digikey"/>
+    <hyperlink ref="O3" r:id="rId3" display="LCSC"/>
+    <hyperlink ref="O4" r:id="rId4" display="LCSC"/>
+    <hyperlink ref="O5" r:id="rId5" display="LCSC"/>
+    <hyperlink ref="O6" r:id="rId6" display="LCSC"/>
+    <hyperlink ref="O7" r:id="rId7" display="LCSC"/>
+    <hyperlink ref="O10" r:id="rId8" display="LCSC"/>
+    <hyperlink ref="O12" r:id="rId9" display="LCSC"/>
+    <hyperlink ref="O13" r:id="rId10" display="LCSC"/>
+    <hyperlink ref="O14" r:id="rId11" display="LCSC"/>
+    <hyperlink ref="O15" r:id="rId12" display="LCSC"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:R17"/>
@@ -2536,7 +3431,7 @@
       <c r="Q1" s="13"/>
       <c r="R1" s="13"/>
     </row>
-    <row r="2" spans="1:18">
+    <row r="2" ht="15.75" spans="1:18">
       <c r="A2" s="2"/>
       <c r="B2" s="5" t="s">
         <v>0</v>
@@ -2572,19 +3467,19 @@
         <v>10</v>
       </c>
       <c r="M2" s="5" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="N2" s="14" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="O2" s="5" t="s">
         <v>13</v>
       </c>
       <c r="P2" s="15" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="Q2" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="R2" s="5" t="s">
         <v>16</v>

</xml_diff>